<commit_message>
SAF :: Work in Progress
</commit_message>
<xml_diff>
--- a/.docs/data/SAF Process and Validation Consolidated Notes.xlsx
+++ b/.docs/data/SAF Process and Validation Consolidated Notes.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12180" tabRatio="563"/>
+    <workbookView windowWidth="28800" windowHeight="12180" tabRatio="563" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Amy &amp; Rachel SAF Process Notes" sheetId="1" r:id="rId1"/>
@@ -775,7 +775,7 @@
     <numFmt numFmtId="176" formatCode="_-&quot;€&quot;* #,##0.00_-;\-&quot;€&quot;* #,##0.00_-;_-&quot;€&quot;* \-??_-;_-@_-"/>
     <numFmt numFmtId="177" formatCode="_-&quot;€&quot;* #,##0_-;\-&quot;€&quot;* #,##0_-;_-&quot;€&quot;* &quot;-&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="29">
+  <fonts count="28">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -820,13 +820,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <name val="Aptos Narrow"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -992,7 +985,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="38">
+  <fills count="40">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1007,6 +1000,24 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.25"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.25"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="3" tint="0.499984740745262"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -1014,12 +1025,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.25"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1425,85 +1430,79 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="9" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="9" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1512,10 +1511,10 @@
     <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1524,10 +1523,10 @@
     <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1536,10 +1535,10 @@
     <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1548,10 +1547,10 @@
     <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1560,17 +1559,23 @@
     <xf numFmtId="0" fontId="25" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="25" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1619,25 +1624,37 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -1664,16 +1681,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1779,8 +1796,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4969510" y="561975"/>
-          <a:ext cx="2465705" cy="2447290"/>
+          <a:off x="4969510" y="590550"/>
+          <a:ext cx="2465705" cy="2228215"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1817,8 +1834,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4880610" y="3388360"/>
-          <a:ext cx="1485900" cy="1804035"/>
+          <a:off x="4880610" y="3216910"/>
+          <a:ext cx="1485900" cy="1727835"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1855,8 +1872,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6298565" y="3307080"/>
-          <a:ext cx="1525905" cy="1837690"/>
+          <a:off x="6298565" y="3135630"/>
+          <a:ext cx="1525905" cy="1761490"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1893,8 +1910,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4979670" y="13991590"/>
-          <a:ext cx="1904365" cy="1579880"/>
+          <a:off x="4979670" y="13353415"/>
+          <a:ext cx="1904365" cy="1303655"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2185,81 +2202,81 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A5:C121"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="19" style="26" customWidth="1"/>
+    <col min="1" max="1" width="19" style="30" customWidth="1"/>
     <col min="2" max="2" width="43.7083333333333" style="1" customWidth="1"/>
-    <col min="3" max="3" width="64.1416666666667" style="26" customWidth="1"/>
-    <col min="4" max="16384" width="9" style="26"/>
+    <col min="3" max="3" width="64.1416666666667" style="30" customWidth="1"/>
+    <col min="4" max="16384" width="9" style="30"/>
   </cols>
   <sheetData>
-    <row r="5" spans="1:1">
-      <c r="A5" s="27" t="s">
+    <row r="5" ht="15" spans="1:1">
+      <c r="A5" s="31" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="7" ht="40.5" spans="1:2">
-      <c r="A7" s="28" t="s">
+    <row r="7" ht="42.75" spans="1:2">
+      <c r="A7" s="32" t="s">
         <v>1</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="8" ht="67.5" spans="1:2">
-      <c r="A8" s="29"/>
+    <row r="8" ht="42.75" spans="1:2">
+      <c r="A8" s="33"/>
       <c r="B8" s="5" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="16" spans="1:2">
-      <c r="A16" s="28" t="s">
+      <c r="A16" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="B16" s="30" t="s">
+      <c r="B16" s="34" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="17" ht="81" spans="1:2">
-      <c r="A17" s="29"/>
-      <c r="B17" s="30" t="s">
+    <row r="17" ht="71.25" spans="1:2">
+      <c r="A17" s="33"/>
+      <c r="B17" s="34" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="18" spans="1:2">
-      <c r="A18" s="31" t="s">
+      <c r="A18" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="B18" s="31"/>
-    </row>
-    <row r="22" spans="1:1">
-      <c r="A22" s="27" t="s">
+      <c r="B18" s="35"/>
+    </row>
+    <row r="22" ht="15" spans="1:1">
+      <c r="A22" s="31" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="24" ht="40.5" spans="1:2">
-      <c r="A24" s="31" t="s">
+    <row r="24" ht="42.75" spans="1:2">
+      <c r="A24" s="35" t="s">
         <v>9</v>
       </c>
       <c r="B24" s="5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="25" ht="67.5" spans="1:2">
-      <c r="A25" s="31" t="s">
+    <row r="25" ht="71.25" spans="1:2">
+      <c r="A25" s="35" t="s">
         <v>11</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="28" spans="1:1">
-      <c r="A28" s="27" t="s">
+    <row r="28" ht="15" spans="1:1">
+      <c r="A28" s="31" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="30" spans="1:2">
-      <c r="A30" s="31" t="s">
+      <c r="A30" s="35" t="s">
         <v>14</v>
       </c>
       <c r="B30" s="5" t="s">
@@ -2267,7 +2284,7 @@
       </c>
     </row>
     <row r="31" spans="1:2">
-      <c r="A31" s="31" t="s">
+      <c r="A31" s="35" t="s">
         <v>16</v>
       </c>
       <c r="B31" s="5" t="s">
@@ -2275,161 +2292,161 @@
       </c>
     </row>
     <row r="32" spans="1:3">
-      <c r="A32" s="31" t="s">
+      <c r="A32" s="35" t="s">
         <v>17</v>
       </c>
       <c r="B32" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C32" s="26" t="s">
+      <c r="C32" s="30" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="33" spans="1:3">
-      <c r="A33" s="31" t="s">
+      <c r="A33" s="35" t="s">
         <v>19</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C33" s="26" t="s">
+      <c r="C33" s="30" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="34" spans="1:3">
-      <c r="A34" s="31" t="s">
+      <c r="A34" s="35" t="s">
         <v>20</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C34" s="26" t="s">
+      <c r="C34" s="30" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="37" spans="1:1">
-      <c r="A37" s="27" t="s">
+    <row r="37" ht="15" spans="1:1">
+      <c r="A37" s="31" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="39" ht="27" spans="1:2">
-      <c r="A39" s="28" t="s">
+    <row r="39" spans="1:2">
+      <c r="A39" s="32" t="s">
         <v>23</v>
       </c>
       <c r="B39" s="5" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="40" ht="40.5" spans="1:2">
-      <c r="A40" s="32"/>
+    <row r="40" ht="28.5" spans="1:2">
+      <c r="A40" s="36"/>
       <c r="B40" s="5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="41" ht="40.5" spans="1:2">
-      <c r="A41" s="32"/>
+    <row r="41" ht="28.5" spans="1:2">
+      <c r="A41" s="36"/>
       <c r="B41" s="5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="42" ht="40.5" spans="1:3">
-      <c r="A42" s="32"/>
+    <row r="42" ht="28.5" spans="1:3">
+      <c r="A42" s="36"/>
       <c r="B42" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="C42" s="26" t="s">
+      <c r="C42" s="30" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="43" ht="27" spans="1:2">
-      <c r="A43" s="29"/>
+    <row r="43" ht="28.5" spans="1:2">
+      <c r="A43" s="33"/>
       <c r="B43" s="5" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="45" ht="40.5" spans="1:3">
-      <c r="A45" s="28" t="s">
+    <row r="45" ht="42.75" spans="1:3">
+      <c r="A45" s="32" t="s">
         <v>30</v>
       </c>
       <c r="B45" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="C45" s="26" t="s">
+      <c r="C45" s="30" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="46" ht="27" spans="1:3">
-      <c r="A46" s="29"/>
+    <row r="46" ht="28.5" spans="1:3">
+      <c r="A46" s="33"/>
       <c r="B46" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C46" s="26" t="s">
+      <c r="C46" s="30" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="47" ht="67.5" spans="1:3">
-      <c r="A47" s="28" t="s">
+    <row r="47" ht="57" spans="1:3">
+      <c r="A47" s="32" t="s">
         <v>35</v>
       </c>
       <c r="B47" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="C47" s="26" t="s">
+      <c r="C47" s="30" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="48" ht="27" spans="1:2">
-      <c r="A48" s="29" t="s">
+    <row r="48" ht="28.5" spans="1:2">
+      <c r="A48" s="33" t="s">
         <v>35</v>
       </c>
       <c r="B48" s="5" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="50" ht="27" spans="1:2">
-      <c r="A50" s="33" t="s">
+    <row r="50" spans="1:2">
+      <c r="A50" s="37" t="s">
         <v>37</v>
       </c>
-      <c r="B50" s="34" t="s">
+      <c r="B50" s="38" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="51" ht="40.5" spans="1:2">
-      <c r="A51" s="35"/>
-      <c r="B51" s="34" t="s">
+    <row r="51" ht="42.75" spans="1:2">
+      <c r="A51" s="39"/>
+      <c r="B51" s="38" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="52" ht="40.5" spans="1:2">
-      <c r="A52" s="36"/>
-      <c r="B52" s="34" t="s">
+    <row r="52" ht="28.5" spans="1:2">
+      <c r="A52" s="40"/>
+      <c r="B52" s="38" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="56" ht="67.5" spans="1:2">
-      <c r="A56" s="28" t="s">
+    <row r="56" ht="57" spans="1:2">
+      <c r="A56" s="32" t="s">
         <v>41</v>
       </c>
       <c r="B56" s="5" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="57" ht="81" spans="1:2">
-      <c r="A57" s="28" t="s">
+    <row r="57" ht="85.5" spans="1:2">
+      <c r="A57" s="32" t="s">
         <v>43</v>
       </c>
-      <c r="B57" s="30" t="s">
+      <c r="B57" s="34" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="58" ht="27" spans="1:2">
-      <c r="A58" s="29"/>
-      <c r="B58" s="37" t="s">
+    <row r="58" ht="28.5" spans="1:2">
+      <c r="A58" s="33"/>
+      <c r="B58" s="41" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="61" spans="1:2">
-      <c r="A61" s="31" t="s">
+      <c r="A61" s="35" t="s">
         <v>46</v>
       </c>
       <c r="B61" s="5" t="s">
@@ -2437,92 +2454,92 @@
       </c>
     </row>
     <row r="64" spans="1:1">
-      <c r="A64" s="26" t="s">
+      <c r="A64" s="30" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="65" ht="67.5" spans="1:3">
-      <c r="A65" s="31" t="s">
+    <row r="65" ht="57" spans="1:3">
+      <c r="A65" s="35" t="s">
         <v>49</v>
       </c>
       <c r="B65" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="C65" s="26" t="s">
+      <c r="C65" s="30" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="66" ht="27" spans="1:3">
-      <c r="A66" s="31" t="s">
+    <row r="66" ht="28.5" spans="1:3">
+      <c r="A66" s="35" t="s">
         <v>49</v>
       </c>
       <c r="B66" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C66" s="26" t="s">
+      <c r="C66" s="30" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="68" ht="40.5" spans="1:2">
-      <c r="A68" s="31" t="s">
+    <row r="68" ht="42.75" spans="1:2">
+      <c r="A68" s="35" t="s">
         <v>52</v>
       </c>
       <c r="B68" s="5" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="69" ht="27" spans="1:2">
-      <c r="A69" s="31" t="s">
+    <row r="69" ht="28.5" spans="1:2">
+      <c r="A69" s="35" t="s">
         <v>52</v>
       </c>
       <c r="B69" s="5" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="72" spans="1:1">
-      <c r="A72" s="27" t="s">
+    <row r="72" ht="15" spans="1:1">
+      <c r="A72" s="31" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="74" spans="1:1">
-      <c r="A74" s="26" t="s">
+      <c r="A74" s="30" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="75" ht="40.5" spans="1:2">
-      <c r="A75" s="31" t="s">
+    <row r="75" ht="28.5" spans="1:2">
+      <c r="A75" s="35" t="s">
         <v>49</v>
       </c>
       <c r="B75" s="5" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="76" ht="27" spans="1:2">
-      <c r="A76" s="31" t="s">
+    <row r="76" ht="28.5" spans="1:2">
+      <c r="A76" s="35" t="s">
         <v>49</v>
       </c>
       <c r="B76" s="5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="77" ht="27" spans="1:2">
-      <c r="A77" s="31" t="s">
+    <row r="77" ht="28.5" spans="1:2">
+      <c r="A77" s="35" t="s">
         <v>49</v>
       </c>
       <c r="B77" s="5" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="79" ht="27" spans="1:2">
-      <c r="A79" s="31" t="s">
+    <row r="79" ht="28.5" spans="1:2">
+      <c r="A79" s="35" t="s">
         <v>60</v>
       </c>
       <c r="B79" s="5" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="80" ht="108" spans="1:2">
-      <c r="A80" s="31" t="s">
+    <row r="80" ht="85.5" spans="1:2">
+      <c r="A80" s="35" t="s">
         <v>62</v>
       </c>
       <c r="B80" s="5" t="s">
@@ -2530,91 +2547,91 @@
       </c>
     </row>
     <row r="82" spans="1:3">
-      <c r="A82" s="31" t="s">
+      <c r="A82" s="35" t="s">
         <v>64</v>
       </c>
       <c r="B82" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="C82" s="26" t="s">
+      <c r="C82" s="30" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="85" spans="1:1">
-      <c r="A85" s="27" t="s">
+    <row r="85" ht="15" spans="1:1">
+      <c r="A85" s="31" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="87" s="25" customFormat="1" ht="40.5" spans="1:2">
-      <c r="A87" s="38" t="s">
+    <row r="87" s="29" customFormat="1" ht="42.75" spans="1:2">
+      <c r="A87" s="42" t="s">
         <v>67</v>
       </c>
-      <c r="B87" s="39" t="s">
+      <c r="B87" s="43" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="88" s="25" customFormat="1" spans="2:2">
-      <c r="B88" s="40"/>
-    </row>
-    <row r="89" s="25" customFormat="1" ht="54" spans="1:2">
-      <c r="A89" s="38" t="s">
+    <row r="88" s="29" customFormat="1" spans="2:2">
+      <c r="B88" s="44"/>
+    </row>
+    <row r="89" s="29" customFormat="1" ht="42.75" spans="1:2">
+      <c r="A89" s="42" t="s">
         <v>69</v>
       </c>
-      <c r="B89" s="39" t="s">
+      <c r="B89" s="43" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="92" ht="27" spans="1:2">
-      <c r="A92" s="28" t="s">
+    <row r="92" spans="1:2">
+      <c r="A92" s="32" t="s">
         <v>71</v>
       </c>
-      <c r="B92" s="30" t="s">
+      <c r="B92" s="34" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="93" ht="27" spans="1:2">
-      <c r="A93" s="32"/>
-      <c r="B93" s="30" t="s">
+    <row r="93" ht="28.5" spans="1:2">
+      <c r="A93" s="36"/>
+      <c r="B93" s="34" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="94" ht="40.5" spans="1:2">
-      <c r="A94" s="32"/>
-      <c r="B94" s="30" t="s">
+    <row r="94" ht="42.75" spans="1:2">
+      <c r="A94" s="36"/>
+      <c r="B94" s="34" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="95" spans="1:2">
-      <c r="A95" s="29"/>
-      <c r="B95" s="30" t="s">
+      <c r="A95" s="33"/>
+      <c r="B95" s="34" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="97" spans="1:2">
-      <c r="A97" s="28" t="s">
+      <c r="A97" s="32" t="s">
         <v>71</v>
       </c>
-      <c r="B97" s="30" t="s">
+      <c r="B97" s="34" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="98" ht="148.5" spans="1:3">
-      <c r="A98" s="29"/>
-      <c r="B98" s="30" t="s">
+    <row r="98" ht="99.75" spans="1:3">
+      <c r="A98" s="33"/>
+      <c r="B98" s="34" t="s">
         <v>77</v>
       </c>
       <c r="C98" s="1"/>
     </row>
     <row r="100" spans="1:2">
-      <c r="A100" s="31" t="s">
+      <c r="A100" s="35" t="s">
         <v>78</v>
       </c>
       <c r="B100" s="5" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="102" ht="40.5" spans="1:2">
-      <c r="A102" s="31" t="s">
+    <row r="102" ht="28.5" spans="1:2">
+      <c r="A102" s="35" t="s">
         <v>80</v>
       </c>
       <c r="B102" s="5" t="s">
@@ -2622,70 +2639,70 @@
       </c>
     </row>
     <row r="106" spans="1:2">
-      <c r="A106" s="21" t="s">
+      <c r="A106" s="22" t="s">
         <v>82</v>
       </c>
-      <c r="B106" s="21"/>
+      <c r="B106" s="22"/>
     </row>
     <row r="107" spans="1:2">
-      <c r="A107" s="21"/>
-      <c r="B107" s="21"/>
+      <c r="A107" s="22"/>
+      <c r="B107" s="22"/>
     </row>
     <row r="108" spans="1:2">
-      <c r="A108" s="21"/>
-      <c r="B108" s="21"/>
+      <c r="A108" s="22"/>
+      <c r="B108" s="22"/>
     </row>
     <row r="109" spans="1:2">
-      <c r="A109" s="21"/>
-      <c r="B109" s="21"/>
+      <c r="A109" s="22"/>
+      <c r="B109" s="22"/>
     </row>
     <row r="110" spans="1:2">
-      <c r="A110" s="21"/>
-      <c r="B110" s="21"/>
+      <c r="A110" s="22"/>
+      <c r="B110" s="22"/>
     </row>
     <row r="111" spans="1:2">
-      <c r="A111" s="21"/>
-      <c r="B111" s="21"/>
+      <c r="A111" s="22"/>
+      <c r="B111" s="22"/>
     </row>
     <row r="112" spans="1:2">
-      <c r="A112" s="21"/>
-      <c r="B112" s="21"/>
+      <c r="A112" s="22"/>
+      <c r="B112" s="22"/>
     </row>
     <row r="113" spans="1:2">
-      <c r="A113" s="21"/>
-      <c r="B113" s="21"/>
+      <c r="A113" s="22"/>
+      <c r="B113" s="22"/>
     </row>
     <row r="114" spans="1:2">
-      <c r="A114" s="21"/>
-      <c r="B114" s="21"/>
+      <c r="A114" s="22"/>
+      <c r="B114" s="22"/>
     </row>
     <row r="115" spans="1:2">
-      <c r="A115" s="21"/>
-      <c r="B115" s="21"/>
+      <c r="A115" s="22"/>
+      <c r="B115" s="22"/>
     </row>
     <row r="116" spans="1:2">
-      <c r="A116" s="21"/>
-      <c r="B116" s="21"/>
+      <c r="A116" s="22"/>
+      <c r="B116" s="22"/>
     </row>
     <row r="117" spans="1:2">
-      <c r="A117" s="21"/>
-      <c r="B117" s="21"/>
+      <c r="A117" s="22"/>
+      <c r="B117" s="22"/>
     </row>
     <row r="118" spans="1:2">
-      <c r="A118" s="21"/>
-      <c r="B118" s="21"/>
+      <c r="A118" s="22"/>
+      <c r="B118" s="22"/>
     </row>
     <row r="119" spans="1:2">
-      <c r="A119" s="21"/>
-      <c r="B119" s="21"/>
+      <c r="A119" s="22"/>
+      <c r="B119" s="22"/>
     </row>
     <row r="120" spans="1:2">
-      <c r="A120" s="21"/>
-      <c r="B120" s="21"/>
+      <c r="A120" s="22"/>
+      <c r="B120" s="22"/>
     </row>
     <row r="121" spans="1:2">
-      <c r="A121" s="21"/>
-      <c r="B121" s="21"/>
+      <c r="A121" s="22"/>
+      <c r="B121" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2707,251 +2724,251 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:C22"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="9.14166666666667" style="17"/>
     <col min="2" max="2" width="35.1416666666667" style="17" customWidth="1"/>
-    <col min="3" max="3" width="135" style="18" customWidth="1"/>
-    <col min="4" max="16384" width="9.14166666666667" style="18"/>
+    <col min="3" max="3" width="135" style="19" customWidth="1"/>
+    <col min="4" max="16384" width="9.14166666666667" style="19"/>
   </cols>
   <sheetData>
     <row r="1" s="17" customFormat="1" spans="1:3">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="20" t="s">
         <v>83</v>
       </c>
-      <c r="B1" s="19" t="s">
+      <c r="B1" s="20" t="s">
         <v>84</v>
       </c>
-      <c r="C1" s="19" t="s">
+      <c r="C1" s="20" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="2" ht="40.5" spans="1:3">
-      <c r="A2" s="20" t="s">
+    <row r="2" ht="42.75" spans="1:3">
+      <c r="A2" s="21" t="s">
         <v>86</v>
       </c>
-      <c r="B2" s="20" t="s">
+      <c r="B2" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="22" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="3" ht="40.5" spans="1:3">
-      <c r="A3" s="20" t="s">
+    <row r="3" s="18" customFormat="1" ht="42.75" spans="1:3">
+      <c r="A3" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="C3" s="21" t="s">
+      <c r="C3" s="24" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="4" ht="81" spans="1:3">
-      <c r="A4" s="20" t="s">
+    <row r="4" ht="86.25" spans="1:3">
+      <c r="A4" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="B4" s="20" t="s">
+      <c r="B4" s="25" t="s">
         <v>91</v>
       </c>
-      <c r="C4" s="21" t="s">
+      <c r="C4" s="22" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="5" ht="94.5" spans="1:3">
-      <c r="A5" s="20" t="s">
+    <row r="5" s="18" customFormat="1" ht="99.75" spans="1:3">
+      <c r="A5" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="23" t="s">
         <v>93</v>
       </c>
-      <c r="C5" s="22" t="s">
+      <c r="C5" s="26" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="6" ht="108" spans="1:3">
-      <c r="A6" s="20" t="s">
+    <row r="6" s="18" customFormat="1" ht="114" spans="1:3">
+      <c r="A6" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="B6" s="20" t="s">
+      <c r="B6" s="23" t="s">
         <v>95</v>
       </c>
-      <c r="C6" s="21" t="s">
+      <c r="C6" s="24" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="7" ht="121.5" spans="1:3">
-      <c r="A7" s="20" t="s">
+    <row r="7" s="18" customFormat="1" ht="114" spans="1:3">
+      <c r="A7" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="B7" s="20" t="s">
+      <c r="B7" s="23" t="s">
         <v>97</v>
       </c>
-      <c r="C7" s="21" t="s">
+      <c r="C7" s="24" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="8" ht="67.5" spans="1:3">
-      <c r="A8" s="20" t="s">
+    <row r="8" s="18" customFormat="1" ht="71.25" spans="1:3">
+      <c r="A8" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="23" t="s">
         <v>99</v>
       </c>
-      <c r="C8" s="22" t="s">
+      <c r="C8" s="26" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="9" ht="27" spans="1:3">
-      <c r="A9" s="20" t="s">
+    <row r="9" ht="28.5" spans="1:3">
+      <c r="A9" s="21" t="s">
         <v>86</v>
       </c>
-      <c r="B9" s="20" t="s">
+      <c r="B9" s="21" t="s">
         <v>101</v>
       </c>
-      <c r="C9" s="21" t="s">
+      <c r="C9" s="22" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="10" ht="27" spans="1:3">
-      <c r="A10" s="20" t="s">
+    <row r="10" s="18" customFormat="1" ht="28.5" spans="1:3">
+      <c r="A10" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="B10" s="20" t="s">
+      <c r="B10" s="23" t="s">
         <v>103</v>
       </c>
-      <c r="C10" s="21" t="s">
+      <c r="C10" s="24" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="11" ht="27" spans="1:3">
-      <c r="A11" s="20" t="s">
+    <row r="11" s="18" customFormat="1" ht="28.5" spans="1:3">
+      <c r="A11" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="B11" s="20" t="s">
+      <c r="B11" s="23" t="s">
         <v>105</v>
       </c>
-      <c r="C11" s="21" t="s">
+      <c r="C11" s="24" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="12" ht="135" spans="1:3">
-      <c r="A12" s="20" t="s">
+    <row r="12" s="18" customFormat="1" ht="142.5" spans="1:3">
+      <c r="A12" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="B12" s="20" t="s">
+      <c r="B12" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="22" t="s">
+      <c r="C12" s="26" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="13" ht="27" spans="1:3">
-      <c r="A13" s="20" t="s">
+    <row r="13" ht="28.5" spans="1:3">
+      <c r="A13" s="21" t="s">
         <v>86</v>
       </c>
-      <c r="B13" s="20" t="s">
+      <c r="B13" s="21" t="s">
         <v>108</v>
       </c>
-      <c r="C13" s="21" t="s">
+      <c r="C13" s="22" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="14" spans="1:3">
-      <c r="A14" s="20" t="s">
+      <c r="A14" s="27" t="s">
         <v>86</v>
       </c>
-      <c r="B14" s="23" t="s">
+      <c r="B14" s="27" t="s">
         <v>110</v>
       </c>
-      <c r="C14" s="24"/>
-    </row>
-    <row r="15" ht="148.5" spans="1:3">
-      <c r="A15" s="20" t="s">
+      <c r="C14" s="28"/>
+    </row>
+    <row r="15" ht="156.75" spans="1:3">
+      <c r="A15" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="B15" s="20" t="s">
+      <c r="B15" s="25" t="s">
         <v>111</v>
       </c>
-      <c r="C15" s="21" t="s">
+      <c r="C15" s="22" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="16" ht="94.5" spans="1:3">
-      <c r="A16" s="20" t="s">
+    <row r="16" ht="99.75" spans="1:3">
+      <c r="A16" s="21" t="s">
         <v>86</v>
       </c>
-      <c r="B16" s="20" t="s">
+      <c r="B16" s="21" t="s">
         <v>113</v>
       </c>
-      <c r="C16" s="21" t="s">
+      <c r="C16" s="22" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="17" ht="40.5" spans="1:3">
-      <c r="A17" s="20" t="s">
+    <row r="17" ht="42.75" spans="1:3">
+      <c r="A17" s="21" t="s">
         <v>86</v>
       </c>
-      <c r="B17" s="20" t="s">
+      <c r="B17" s="21" t="s">
         <v>115</v>
       </c>
-      <c r="C17" s="21" t="s">
+      <c r="C17" s="22" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="18" ht="40.5" spans="1:3">
-      <c r="A18" s="20" t="s">
+    <row r="18" ht="45" spans="1:3">
+      <c r="A18" s="21" t="s">
         <v>86</v>
       </c>
-      <c r="B18" s="20" t="s">
+      <c r="B18" s="21" t="s">
         <v>117</v>
       </c>
-      <c r="C18" s="21" t="s">
+      <c r="C18" s="22" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="19" ht="67.5" spans="1:3">
-      <c r="A19" s="20" t="s">
+    <row r="19" ht="71.25" spans="1:3">
+      <c r="A19" s="21" t="s">
         <v>86</v>
       </c>
-      <c r="B19" s="20" t="s">
+      <c r="B19" s="21" t="s">
         <v>108</v>
       </c>
-      <c r="C19" s="21" t="s">
+      <c r="C19" s="22" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="20" ht="94.5" spans="1:3">
-      <c r="A20" s="20" t="s">
+    <row r="20" ht="99.75" spans="1:3">
+      <c r="A20" s="21" t="s">
         <v>86</v>
       </c>
-      <c r="B20" s="20" t="s">
+      <c r="B20" s="21" t="s">
         <v>120</v>
       </c>
-      <c r="C20" s="21" t="s">
+      <c r="C20" s="22" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="21" ht="270" spans="1:3">
-      <c r="A21" s="20" t="s">
+    <row r="21" ht="243" spans="1:3">
+      <c r="A21" s="21" t="s">
         <v>86</v>
       </c>
-      <c r="B21" s="20" t="s">
+      <c r="B21" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="C21" s="21" t="s">
+      <c r="C21" s="22" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="22" ht="27" spans="1:3">
-      <c r="A22" s="20" t="s">
+    <row r="22" ht="28.5" spans="1:3">
+      <c r="A22" s="21" t="s">
         <v>86</v>
       </c>
-      <c r="B22" s="20" t="s">
+      <c r="B22" s="21" t="s">
         <v>124</v>
       </c>
-      <c r="C22" s="21" t="s">
+      <c r="C22" s="22" t="s">
         <v>125</v>
       </c>
     </row>
@@ -2971,19 +2988,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:B47"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="138.141666666667" style="1" customWidth="1"/>
     <col min="2" max="2" width="108.566666666667" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9.14166666666667" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" ht="15" spans="1:1">
       <c r="A1" s="7" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="2" ht="202.5" spans="1:2">
+    <row r="2" ht="213.75" spans="1:2">
       <c r="A2" s="8" t="s">
         <v>127</v>
       </c>
@@ -2995,25 +3012,25 @@
       </c>
       <c r="B3" s="5"/>
     </row>
-    <row r="4" ht="40.5" spans="1:2">
+    <row r="4" ht="42.75" spans="1:2">
       <c r="A4" s="8" t="s">
         <v>129</v>
       </c>
       <c r="B4" s="5"/>
     </row>
-    <row r="5" ht="67.5" spans="1:2">
+    <row r="5" ht="42.75" spans="1:2">
       <c r="A5" s="8" t="s">
         <v>130</v>
       </c>
       <c r="B5" s="5"/>
     </row>
-    <row r="6" ht="27" spans="1:2">
+    <row r="6" ht="28.5" spans="1:2">
       <c r="A6" s="8" t="s">
         <v>131</v>
       </c>
       <c r="B6" s="5"/>
     </row>
-    <row r="7" ht="54" spans="1:2">
+    <row r="7" ht="57" spans="1:2">
       <c r="A7" s="8" t="s">
         <v>132</v>
       </c>
@@ -3022,13 +3039,13 @@
     <row r="8" spans="2:2">
       <c r="B8" s="5"/>
     </row>
-    <row r="9" ht="14.25" spans="1:2">
+    <row r="9" ht="15.75" spans="1:2">
       <c r="A9" s="9" t="s">
         <v>133</v>
       </c>
       <c r="B9" s="5"/>
     </row>
-    <row r="10" ht="42.75" spans="1:2">
+    <row r="10" ht="45" spans="1:2">
       <c r="A10" s="10" t="s">
         <v>134</v>
       </c>
@@ -3048,7 +3065,7 @@
       <c r="A13" s="11"/>
       <c r="B13" s="12"/>
     </row>
-    <row r="14" ht="14.25" spans="1:2">
+    <row r="14" ht="15" spans="1:2">
       <c r="A14" s="13" t="s">
         <v>30</v>
       </c>
@@ -3056,7 +3073,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="15" ht="14.25" spans="1:2">
+    <row r="15" ht="15" spans="1:2">
       <c r="A15" s="15" t="s">
         <v>137</v>
       </c>
@@ -3064,7 +3081,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="16" ht="14.25" spans="1:2">
+    <row r="16" ht="15" spans="1:2">
       <c r="A16" s="15" t="s">
         <v>139</v>
       </c>
@@ -3072,7 +3089,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="17" ht="14.25" spans="1:2">
+    <row r="17" ht="15" spans="1:2">
       <c r="A17" s="15"/>
       <c r="B17" s="14"/>
     </row>
@@ -3082,7 +3099,7 @@
       </c>
       <c r="B18" s="14"/>
     </row>
-    <row r="19" ht="14.25" spans="1:2">
+    <row r="19" ht="15" spans="1:2">
       <c r="A19" s="15" t="s">
         <v>142</v>
       </c>
@@ -3090,7 +3107,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="20" ht="14.25" spans="1:2">
+    <row r="20" ht="15" spans="1:2">
       <c r="A20" s="15" t="s">
         <v>144</v>
       </c>
@@ -3098,19 +3115,19 @@
         <v>145</v>
       </c>
     </row>
-    <row r="21" ht="14.25" spans="1:2">
+    <row r="21" ht="15" spans="1:2">
       <c r="A21" s="15"/>
       <c r="B21" s="14" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="22" ht="14.25" spans="1:2">
+    <row r="22" ht="15" spans="1:2">
       <c r="A22" s="15"/>
       <c r="B22" s="14" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="23" ht="14.25" spans="1:2">
+    <row r="23" ht="15" spans="1:2">
       <c r="A23" s="15" t="s">
         <v>148</v>
       </c>
@@ -3118,11 +3135,11 @@
         <v>149</v>
       </c>
     </row>
-    <row r="24" ht="14.25" spans="1:2">
+    <row r="24" ht="15" spans="1:2">
       <c r="A24" s="15"/>
       <c r="B24" s="14"/>
     </row>
-    <row r="25" ht="14.25" spans="1:2">
+    <row r="25" ht="15" spans="1:2">
       <c r="A25" s="15"/>
       <c r="B25" s="14"/>
     </row>
@@ -3134,7 +3151,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="27" ht="14.25" spans="1:2">
+    <row r="27" ht="15" spans="1:2">
       <c r="A27" s="15" t="s">
         <v>30</v>
       </c>
@@ -3142,7 +3159,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="28" ht="14.25" spans="1:2">
+    <row r="28" ht="15" spans="1:2">
       <c r="A28" s="15" t="s">
         <v>153</v>
       </c>
@@ -3150,7 +3167,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="29" ht="14.25" spans="1:2">
+    <row r="29" ht="15" spans="1:2">
       <c r="A29" s="15" t="s">
         <v>144</v>
       </c>
@@ -3158,19 +3175,19 @@
         <v>145</v>
       </c>
     </row>
-    <row r="30" ht="14.25" spans="1:2">
+    <row r="30" ht="15" spans="1:2">
       <c r="A30" s="15"/>
       <c r="B30" s="14" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="31" ht="14.25" spans="1:2">
+    <row r="31" ht="15" spans="1:2">
       <c r="A31" s="15"/>
       <c r="B31" s="14" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="32" ht="14.25" spans="1:2">
+    <row r="32" ht="15" spans="1:2">
       <c r="A32" s="15" t="s">
         <v>148</v>
       </c>
@@ -3250,7 +3267,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="5" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelRow="5" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="50.2833333333333" style="1" customWidth="1"/>
     <col min="2" max="2" width="22.5666666666667" style="2" customWidth="1"/>
@@ -3258,7 +3275,7 @@
     <col min="4" max="16384" width="9.14166666666667" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40.5" spans="1:3">
+    <row r="1" ht="45" spans="1:3">
       <c r="A1" s="3" t="s">
         <v>156</v>
       </c>

</xml_diff>